<commit_message>
Complete Milestone 4 dashboard reporting and E2E validation
</commit_message>
<xml_diff>
--- a/Agile/Agile_Template_v0.1.xlsx
+++ b/Agile/Agile_Template_v0.1.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="97" documentId="11_779D2F40EFDA50A0129A453F3B61210D141A5D77" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB551473-15E0-4B40-93E0-7C2E54AA4702}"/>
   <bookViews>
-    <workbookView xWindow="10260" yWindow="2472" windowWidth="12420" windowHeight="8880" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10260" yWindow="2472" windowWidth="12420" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Product Backlog" sheetId="1" r:id="rId1"/>
@@ -514,6 +514,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>